<commit_message>
checkpoint: preserve pre-HKT premium monitor baseline
</commit_message>
<xml_diff>
--- a/database for armmac/outputs/01a03c21-40ce-7230-8082-fa2313f6d1c6/TGW_Mac_API_验收台账.xlsx
+++ b/database for armmac/outputs/01a03c21-40ce-7230-8082-fa2313f6d1c6/TGW_Mac_API_验收台账.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="R665ba1811fc14ee6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="接口验收" sheetId="2" r:id="R7d8de52ee3434d3b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="功能号目录" sheetId="3" r:id="Rf8aa403634bd4c60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据结构" sheetId="4" r:id="R3726d094c8dd4ff3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试批次" sheetId="5" r:id="R38201a1de46c4acd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="状态字典" sheetId="6" r:id="Ra8d955a0bb1a4c72"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="R273dd54d805e437f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="接口验收" sheetId="2" r:id="R57f5925067614631"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="功能号目录" sheetId="3" r:id="R49b47741b8674a58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据结构" sheetId="4" r:id="R9161ad95b9294acf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试批次" sheetId="5" r:id="R699adb59e6454bad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="状态字典" sheetId="6" r:id="R9afe96b6ca8c4b22"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -625,10 +625,10 @@
         <x:v>SZSE ETF L1 历史</x:v>
       </x:c>
       <x:c r="G6" s="18" t="str">
-        <x:v>CHANGES_REQUESTED</x:v>
+        <x:v>LIVE_ALIGNED</x:v>
       </x:c>
       <x:c r="H6" s="18" t="str">
-        <x:v>补错误码/空数据/异步语义</x:v>
+        <x:v>已完成错误码/异步合约；余多包异步交付与其它市场</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -637,7 +637,7 @@
       </x:c>
       <x:c r="B7" s="18" t="n">
         <x:f>COUNTIF('接口验收'!$J$5:$J$168,"LIVE_ALIGNED")</x:f>
-        <x:v>19</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="D7" s="18" t="n">
         <x:v>2</x:v>
@@ -709,7 +709,7 @@
       </x:c>
       <x:c r="B10" s="18" t="n">
         <x:f>COUNTIF('接口验收'!$J$5:$J$168,"CHANGES_REQUESTED")</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D10" s="18" t="n">
         <x:v>5</x:v>
@@ -757,7 +757,7 @@
       </x:c>
       <x:c r="B12" s="23" t="n">
         <x:f>AVERAGE('接口验收'!$K$5:$K$168)</x:f>
-        <x:v>20.365853658536587</x:v>
+        <x:v>21.524390243902438</x:v>
       </x:c>
       <x:c r="D12" s="18" t="n">
         <x:v>7</x:v>
@@ -3459,10 +3459,10 @@
         <x:v>已有 Mac 子范围证据</x:v>
       </x:c>
       <x:c r="Q36" s="18" t="str">
-        <x:v>LIVE_ALIGNED(daily + weekly + monthly only)：10008→10100，10009→10101，10010→10102；响应 tag 同 wire 周期</x:v>
+        <x:v>LIVE_ALIGNED(daily + weekly + monthly + quarterly + yearly only)：10008→10100，10009→10101，10010→10102，10011→10103，10012→10104（季/年已实捕证明）；响应 tag 同 wire 周期</x:v>
       </x:c>
       <x:c r="R36" s="18" t="str">
-        <x:v>已有 SSE 510300 日线单日、周线单周与月线单月；Linux oracle → wire → Mac → 同参</x:v>
+        <x:v>已有 SSE 510300 日线单日、周线单周、月线单月、季线单季与年线单年；Linux oracle → wire → Mac → 同参</x:v>
       </x:c>
       <x:c r="S36" s="18" t="str">
         <x:v>ReqKline{code[38],market u8,cq_flag u8,cq_date,qj_flag,cyc_type u16,cyc_def,auto_complete,begin/end_date,begin/end_time} pack(1)=71</x:v>
@@ -3477,10 +3477,10 @@
         <x:v>docs/PDF_API_INVENTORY.md</x:v>
       </x:c>
       <x:c r="W36" s="18" t="str">
-        <x:v>已有 SSE 510300 日线单日、周线单周与月线单月</x:v>
+        <x:v>已有 SSE 510300 日线单日、周线单周、月线单月、季线单季与年线单年</x:v>
       </x:c>
       <x:c r="X36" s="18" t="str">
-        <x:v>季/年/分钟族显式拒绝；非零 status（kDataEmpty=-76）转异常未对齐官方错误码返回；备用端点受 1000 accept conn active close 流控</x:v>
+        <x:v>分钟族显式拒绝；非零 status（kDataEmpty=-76）转异常未对齐官方错误码返回；备用端点受 1000 accept conn active close 流控</x:v>
       </x:c>
       <x:c r="Y36" s="18" t="str"/>
     </x:row>
@@ -3513,15 +3513,17 @@
         <x:v>低</x:v>
       </x:c>
       <x:c r="J37" s="18" t="str">
-        <x:v>CHANGES_REQUESTED</x:v>
+        <x:v>LIVE_ALIGNED</x:v>
       </x:c>
       <x:c r="K37" s="19" t="n">
         <x:f>IFERROR(VLOOKUP(J37,'状态字典'!$A$5:$B$16,2,FALSE),0)</x:f>
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="L37" s="18" t="str"/>
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="L37" s="18" t="str">
+        <x:v>2026-08-26</x:v>
+      </x:c>
       <x:c r="M37" s="18" t="str">
-        <x:v>未执行</x:v>
+        <x:v>已有脱敏证据；严格限于状态所述子范围</x:v>
       </x:c>
       <x:c r="N37" s="18" t="str">
         <x:v>data_type 0/1/2 其余无效；level_type 默认0</x:v>
@@ -3530,10 +3532,10 @@
         <x:v>2026-08-26</x:v>
       </x:c>
       <x:c r="P37" s="18" t="str">
-        <x:v>待实现/复验</x:v>
+        <x:v>已有 Mac 子范围证据</x:v>
       </x:c>
       <x:c r="Q37" s="18" t="str">
-        <x:v>数据/协议已 Linux/Mac 同参（SZSE 159518,data_type=0,level=0,tag 11000）；公开合约 CHANGES_REQUESTED</x:v>
+        <x:v>LIVE_ALIGNED(SZSE ETF L1, data_type=0; sync+async error contract)：数据/协议同参 + 空数据 (None,-76)/异步 (True,None)→(None,-76) 均已 Linux/Mac 同参（2026-08-26）</x:v>
       </x:c>
       <x:c r="R37" s="18" t="str">
         <x:v>已有单日窄窗；Linux oracle → wire → Mac → 同参</x:v>
@@ -3554,7 +3556,7 @@
         <x:v>已有单日窄窗</x:v>
       </x:c>
       <x:c r="X37" s="18" t="str">
-        <x:v>异步 SPI 合约与公开错误语义未验收；data_type=1/2 未取证；市场范围未验</x:v>
+        <x:v>多包异步交付语义未观测；data_type=1/2 未取证；其它市场未验；错误标签映射仅 "DataEmpty" 已捕获</x:v>
       </x:c>
       <x:c r="Y37" s="18" t="str"/>
     </x:row>
@@ -3803,11 +3805,11 @@
         <x:v>低</x:v>
       </x:c>
       <x:c r="J41" s="18" t="str">
-        <x:v>STATIC_MATCHED</x:v>
+        <x:v>ARM_IMPLEMENTED</x:v>
       </x:c>
       <x:c r="K41" s="19" t="n">
         <x:f>IFERROR(VLOOKUP(J41,'状态字典'!$A$5:$B$16,2,FALSE),0)</x:f>
-        <x:v>25</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="L41" s="18" t="str"/>
       <x:c r="M41" s="18" t="str">
@@ -3816,15 +3818,17 @@
       <x:c r="N41" s="18" t="str">
         <x:v>含 2022-08-22 起退市代码</x:v>
       </x:c>
-      <x:c r="O41" s="18" t="str"/>
+      <x:c r="O41" s="18" t="str">
+        <x:v>2026-08-26</x:v>
+      </x:c>
       <x:c r="P41" s="18" t="str">
-        <x:v>待实现/复验</x:v>
+        <x:v>已有实现；待同参 live</x:v>
       </x:c>
       <x:c r="Q41" s="18" t="str">
-        <x:v>STATIC_MATCHED(static contract only)</x:v>
+        <x:v>ARM_IMPLEMENTED</x:v>
       </x:c>
       <x:c r="R41" s="18" t="str">
-        <x:v>全市场一次查询取行数/列型摘要；用异步 SPI 收齐批次；Linux oracle → wire → Mac → 同参</x:v>
+        <x:v>wire 已证：dgw*_query one-shot、ReqGetReduceCodeTable、tag 11103、反引号 6 字段、缺包 ReqGetPackage；Linux -83 与 Mac 缺包超时同因同果（服务端缺第 3 包）；待成功同参闭环；Linux oracle → wire → Mac → 同参</x:v>
       </x:c>
       <x:c r="S41" s="18" t="str">
         <x:v>无入参</x:v>
@@ -3839,10 +3843,10 @@
         <x:v>docs/PDF_API_INVENTORY.md</x:v>
       </x:c>
       <x:c r="W41" s="18" t="str">
-        <x:v>全市场一次查询取行数/列型摘要；用异步 SPI 收齐批次</x:v>
+        <x:v>wire 已证：dgw*_query one-shot、ReqGetReduceCodeTable、tag 11103、反引号 6 字段、缺包 ReqGetPackage；Linux -83 与 Mac 缺包超时同因同果（服务端缺第 3 包）；待成功同参闭环</x:v>
       </x:c>
       <x:c r="X41" s="18" t="str">
-        <x:v>官方同步 wrapper 在首批回调即唤醒且覆盖结果，存在首批竞态；wire method/tag 尚未实测</x:v>
+        <x:v>服务端全市场大表持续缺第 3 包且对补拉无响应，完整 12 包成功样本当前不可得；完成 method（ReqGetComplete/ReqGetCodelistComplete）未证</x:v>
       </x:c>
       <x:c r="Y41" s="18" t="str"/>
     </x:row>
@@ -3875,28 +3879,32 @@
         <x:v>低</x:v>
       </x:c>
       <x:c r="J42" s="18" t="str">
-        <x:v>INVENTORIED</x:v>
+        <x:v>LIVE_ALIGNED</x:v>
       </x:c>
       <x:c r="K42" s="19" t="n">
         <x:f>IFERROR(VLOOKUP(J42,'状态字典'!$A$5:$B$16,2,FALSE),0)</x:f>
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="L42" s="18" t="str"/>
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="L42" s="18" t="str">
+        <x:v>2026-08-26</x:v>
+      </x:c>
       <x:c r="M42" s="18" t="str">
-        <x:v>未执行</x:v>
+        <x:v>已有脱敏证据；严格限于状态所述子范围</x:v>
       </x:c>
       <x:c r="N42" s="18" t="str">
         <x:v>market kNone=全市场；支持 SSE/SZSE/NEEQ</x:v>
       </x:c>
-      <x:c r="O42" s="18" t="str"/>
+      <x:c r="O42" s="18" t="str">
+        <x:v>2026-08-26</x:v>
+      </x:c>
       <x:c r="P42" s="18" t="str">
-        <x:v>待实现/复验</x:v>
+        <x:v>已有 Mac 子范围证据</x:v>
       </x:c>
       <x:c r="Q42" s="18" t="str">
-        <x:v>INVENTORIED</x:v>
+        <x:v>LIVE_ALIGNED(SSE single code only)</x:v>
       </x:c>
       <x:c r="R42" s="18" t="str">
-        <x:v>单市场单代码（如 159518.SZSE）；Linux oracle → wire → Mac → 同参</x:v>
+        <x:v>已闭合 SSE 510300 单 item：push 通道 ReqGetCodeTableList、tag "109"、43 字段/MDCodeTableRecord sizeof=555；Linux/Mac 同参 1 行 43 列一致；Linux oracle → wire → Mac → 同参</x:v>
       </x:c>
       <x:c r="S42" s="18" t="str">
         <x:v>SubCodeTableItem{i32 market,char[32] code}</x:v>
@@ -3911,10 +3919,10 @@
         <x:v>docs/PDF_API_INVENTORY.md</x:v>
       </x:c>
       <x:c r="W42" s="18" t="str">
-        <x:v>单市场单代码（如 159518.SZSE）</x:v>
+        <x:v>已闭合 SSE 510300 单 item：push 通道 ReqGetCodeTableList、tag "109"、43 字段/MDCodeTableRecord sizeof=555；Linux/Mac 同参 1 行 43 列一致</x:v>
       </x:c>
       <x:c r="X42" s="18" t="str">
-        <x:v>返回容器列集合需先 Linux oracle 定形</x:v>
+        <x:v>全市场/多 item/SZSE/NEEQ/空结果/多帧分页未验且显式拒绝</x:v>
       </x:c>
       <x:c r="Y42" s="18" t="str"/>
     </x:row>
@@ -3947,28 +3955,32 @@
         <x:v>低</x:v>
       </x:c>
       <x:c r="J43" s="18" t="str">
-        <x:v>INVENTORIED</x:v>
+        <x:v>LIVE_ALIGNED</x:v>
       </x:c>
       <x:c r="K43" s="19" t="n">
         <x:f>IFERROR(VLOOKUP(J43,'状态字典'!$A$5:$B$16,2,FALSE),0)</x:f>
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="L43" s="18" t="str"/>
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="L43" s="18" t="str">
+        <x:v>2026-08-26</x:v>
+      </x:c>
       <x:c r="M43" s="18" t="str">
-        <x:v>未执行</x:v>
+        <x:v>已有脱敏证据；严格限于状态所述子范围</x:v>
       </x:c>
       <x:c r="N43" s="18" t="str">
         <x:v>无</x:v>
       </x:c>
-      <x:c r="O43" s="18" t="str"/>
+      <x:c r="O43" s="18" t="str">
+        <x:v>2026-08-26</x:v>
+      </x:c>
       <x:c r="P43" s="18" t="str">
-        <x:v>待实现/复验</x:v>
+        <x:v>已有 Mac 子范围证据</x:v>
       </x:c>
       <x:c r="Q43" s="18" t="str">
-        <x:v>INVENTORIED</x:v>
+        <x:v>LIVE_ALIGNED(000001 only)</x:v>
       </x:c>
       <x:c r="R43" s="18" t="str">
-        <x:v>000001 单代码；Linux oracle → wire → Mac → 同参</x:v>
+        <x:v>已闭合 000001 单代码：one-shot ReqGetExFactor、tag 11102、5 字段 CSV、double 18 位小数字符串上线、33 行；Linux/Mac 同参（含 cum_factor 单调违例 2 处吻合）；Linux oracle → wire → Mac → 同参</x:v>
       </x:c>
       <x:c r="S43" s="18" t="str">
         <x:v>const char* code</x:v>
@@ -3983,10 +3995,10 @@
         <x:v>docs/PDF_API_INVENTORY.md</x:v>
       </x:c>
       <x:c r="W43" s="18" t="str">
-        <x:v>000001 单代码</x:v>
+        <x:v>已闭合 000001 单代码：one-shot ReqGetExFactor、tag 11102、5 字段 CSV、double 18 位小数字符串上线、33 行；Linux/Mac 同参（含 cum_factor 单调违例 2 处吻合）</x:v>
       </x:c>
       <x:c r="X43" s="18" t="str">
-        <x:v>double 精度与缩放（N38(15)）需 oracle 确认</x:v>
+        <x:v>空结果/非零 status wire 形状未取证；多包未线上观测；异步 SPI 未实现</x:v>
       </x:c>
       <x:c r="Y43" s="18" t="str"/>
     </x:row>
@@ -4679,11 +4691,11 @@
         <x:v>低</x:v>
       </x:c>
       <x:c r="J53" s="18" t="str">
-        <x:v>ARM_IMPLEMENTED</x:v>
+        <x:v>STATIC_MATCHED</x:v>
       </x:c>
       <x:c r="K53" s="19" t="n">
         <x:f>IFERROR(VLOOKUP(J53,'状态字典'!$A$5:$B$16,2,FALSE),0)</x:f>
-        <x:v>70</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="L53" s="18" t="str"/>
       <x:c r="M53" s="18" t="str">
@@ -4692,14 +4704,12 @@
       <x:c r="N53" s="18" t="str">
         <x:v>待逐接口取证</x:v>
       </x:c>
-      <x:c r="O53" s="18" t="str">
-        <x:v>2026-08-26</x:v>
-      </x:c>
+      <x:c r="O53" s="18" t="str"/>
       <x:c r="P53" s="18" t="str">
-        <x:v>已有实现；待同参 live</x:v>
+        <x:v>待实现/复验</x:v>
       </x:c>
       <x:c r="Q53" s="18" t="str">
-        <x:v>ARM_IMPLEMENTED(partial)（GetErrorMsg 仅识别 0）</x:v>
+        <x:v>STATIC_MATCHED(official table)（Mac ErrorCode/GetErrorMsg 已对齐官方 wheel 全表；快照空数据 -76 已线上同参，其余码触发条件未逐项取证）</x:v>
       </x:c>
       <x:c r="R53" s="18" t="str">
         <x:v>按单接口最小只读样本；Linux oracle → wire → Mac → 同参</x:v>
@@ -4720,7 +4730,7 @@
         <x:v>领取单接口任务卡并按工作流闭环</x:v>
       </x:c>
       <x:c r="X53" s="18" t="str">
-        <x:v>Mac 需把非零 status 对齐为官方错误码语义而非异常</x:v>
+        <x:v>其余错误码的线上触发条件需随各接口逐步验证</x:v>
       </x:c>
       <x:c r="Y53" s="18" t="str"/>
     </x:row>
@@ -14484,13 +14494,13 @@
         <x:v>code[16]/symbol[32]/en_name[128]/market u8/type[10]/currency[4]；sizeof=191</x:v>
       </x:c>
       <x:c r="F11" s="18" t="str">
-        <x:v>STATIC_MATCHED</x:v>
+        <x:v>ARM_IMPLEMENTED</x:v>
       </x:c>
       <x:c r="G11" s="18" t="str">
-        <x:v>STATIC_MATCHED(static contract only)</x:v>
+        <x:v>ARM_IMPLEMENTED</x:v>
       </x:c>
       <x:c r="H11" s="18" t="str">
-        <x:v>官方同步 wrapper 有首批竞态；wire 未验</x:v>
+        <x:v>wire 已证（tag 11103 反引号 6 字段）；服务端全市场缺第 3 包阻塞成功同参</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="38" customHeight="1">
@@ -15190,140 +15200,308 @@
       </x:c>
     </x:row>
     <x:row r="14" ht="38" customHeight="1">
-      <x:c r="A14" s="22" t="str">
+      <x:c r="A14" s="18" t="str">
+        <x:v>B-20260826-10</x:v>
+      </x:c>
+      <x:c r="B14" s="18" t="str">
+        <x:v>2026-08-26</x:v>
+      </x:c>
+      <x:c r="C14" s="18" t="str">
+        <x:v>QuerySnapshot</x:v>
+      </x:c>
+      <x:c r="D14" s="18" t="str">
+        <x:v>SZSE ETF L1 同步错误码+异步 SPI（同参复验）</x:v>
+      </x:c>
+      <x:c r="E14" s="18" t="str">
+        <x:v>盘后查询</x:v>
+      </x:c>
+      <x:c r="F14" s="18" t="str">
+        <x:v>空窗 (None,-76)；数据窗 (11行,0)；异步 submit(True,None)+回调(list,11)/(None,-76)</x:v>
+      </x:c>
+      <x:c r="G14" s="18" t="str">
+        <x:v>四场景逐一一致（同步双格式+异步双分支）</x:v>
+      </x:c>
+      <x:c r="H14" s="18" t="str">
+        <x:v>sync+async error contract 一致；多包异步交付仍未观测</x:v>
+      </x:c>
+      <x:c r="I14" s="18" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="J14" s="18" t="str">
+        <x:v>docs/evidence/query_snapshot_error_async_contract.md</x:v>
+      </x:c>
+      <x:c r="K14" s="18" t="str">
+        <x:v>LIVE_ALIGNED</x:v>
+      </x:c>
+      <x:c r="L14" s="18" t="str">
+        <x:v>本轮查询通道3次1000准入回收，低频间隔后恢复；wire 新增 DataEmpty 错误帧形状</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="38" customHeight="1">
+      <x:c r="A15" s="18" t="str">
+        <x:v>B-20260826-11</x:v>
+      </x:c>
+      <x:c r="B15" s="18" t="str">
+        <x:v>2026-08-26</x:v>
+      </x:c>
+      <x:c r="C15" s="18" t="str">
+        <x:v>QueryCodeTable</x:v>
+      </x:c>
+      <x:c r="D15" s="18" t="str">
+        <x:v>互联网全市场 wire 取证 + Mac 实现（ARM）</x:v>
+      </x:c>
+      <x:c r="E15" s="18" t="str">
+        <x:v>盘后查询</x:v>
+      </x:c>
+      <x:c r="F15" s="18" t="str">
+        <x:v>登录成功；sync probe -83 kTimeout（服务端12包缺第3包，ReqGetPackage无响应）；wire: dgw*_query/ReqGetReduceCodeTable/tag11103/反引号6字段/11包共167,269行</x:v>
+      </x:c>
+      <x:c r="G15" s="18" t="str">
+        <x:v>登录成功；缺包超时（同因同果）；dgw2 备用端点 1000 accept conn active close 流控</x:v>
+      </x:c>
+      <x:c r="H15" s="18" t="str">
+        <x:v>无成功同参样本（两侧均被服务端全市场缺包阻塞）；错误语义同因同果</x:v>
+      </x:c>
+      <x:c r="I15" s="18" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="J15" s="18" t="str">
+        <x:v>docs/evidence/query_code_table_live_closure.md</x:v>
+      </x:c>
+      <x:c r="K15" s="18" t="str">
+        <x:v>ARM_IMPLEMENTED</x:v>
+      </x:c>
+      <x:c r="L15" s="18" t="str">
+        <x:v>完成 method 未证；currency/security_type 空白串 trim 待成功样本复核；query_spi 显式拒绝</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="38" customHeight="1">
+      <x:c r="A16" s="18" t="str">
+        <x:v>B-20260826-12</x:v>
+      </x:c>
+      <x:c r="B16" s="18" t="str">
+        <x:v>2026-08-26</x:v>
+      </x:c>
+      <x:c r="C16" s="18" t="str">
+        <x:v>QueryKline</x:v>
+      </x:c>
+      <x:c r="D16" s="18" t="str">
+        <x:v>季线 cyc_type=10011 静态三方契约</x:v>
+      </x:c>
+      <x:c r="E16" s="18" t="str">
+        <x:v>静态核对</x:v>
+      </x:c>
+      <x:c r="F16" s="18" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="G16" s="18" t="str">
+        <x:v>未实现</x:v>
+      </x:c>
+      <x:c r="H16" s="18" t="str">
+        <x:v>PDF/HDR/官方 wrapper 三方一致；MDKLine 11 字段含补列，周期无关</x:v>
+      </x:c>
+      <x:c r="I16" s="18" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="J16" s="18" t="str">
+        <x:v>docs/evidence/query_kline_quarter_static.md</x:v>
+      </x:c>
+      <x:c r="K16" s="18" t="str">
+        <x:v>STATIC_MATCHED</x:v>
+      </x:c>
+      <x:c r="L16" s="18" t="str">
+        <x:v>10011→wire 10103 为外推假设，未实捕，禁止预填实现</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="38" customHeight="1">
+      <x:c r="A17" s="18" t="str">
+        <x:v>B-20260826-13</x:v>
+      </x:c>
+      <x:c r="B17" s="18" t="str">
+        <x:v>2026-08-26</x:v>
+      </x:c>
+      <x:c r="C17" s="18" t="str">
+        <x:v>QueryKline</x:v>
+      </x:c>
+      <x:c r="D17" s="18" t="str">
+        <x:v>季线 cyc_type=10011 Linux/wire/Mac 同参闭环</x:v>
+      </x:c>
+      <x:c r="E17" s="18" t="str">
+        <x:v>盘后查询</x:v>
+      </x:c>
+      <x:c r="F17" s="18" t="str">
+        <x:v>login true、error 0、1行/11列（10 int+1 str）、kline_time 8位、market=[101]；wire 实捕 10011→period_type/tag=10103、单包、ReqGetComplete+正常close</x:v>
+      </x:c>
+      <x:c r="G17" s="18" t="str">
+        <x:v>登录成功、error 0、rows=1、11 列集合/类型与 Linux 完全一致</x:v>
+      </x:c>
+      <x:c r="H17" s="18" t="str">
+        <x:v>quarterly 子范围同参一致</x:v>
+      </x:c>
+      <x:c r="I17" s="18" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="J17" s="18" t="str">
+        <x:v>docs/evidence/query_kline_quarter_live.md</x:v>
+      </x:c>
+      <x:c r="K17" s="18" t="str">
+        <x:v>LIVE_ALIGNED(quarterly only)</x:v>
+      </x:c>
+      <x:c r="L17" s="18" t="str">
+        <x:v>年线/分钟族未验且显式拒绝；季线线上单包样本；跨季多包仅合成覆盖</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="38" customHeight="1">
+      <x:c r="A18" s="18" t="str">
+        <x:v>B-20260826-14</x:v>
+      </x:c>
+      <x:c r="B18" s="18" t="str">
+        <x:v>2026-08-26</x:v>
+      </x:c>
+      <x:c r="C18" s="18" t="str">
+        <x:v>QueryKline</x:v>
+      </x:c>
+      <x:c r="D18" s="18" t="str">
+        <x:v>年线 cyc_type=10012 Linux/wire/Mac 同参闭环</x:v>
+      </x:c>
+      <x:c r="E18" s="18" t="str">
+        <x:v>盘后查询</x:v>
+      </x:c>
+      <x:c r="F18" s="18" t="str">
+        <x:v>login true、error 0、1行/11列；wire 实捕 10012→period_type/tag=10104、单包、ReqGetComplete+正常close</x:v>
+      </x:c>
+      <x:c r="G18" s="18" t="str">
+        <x:v>Mac 首次被 1000 流控回收，低频换备用端点成功后 error 0、rows=1、11 列类型一致</x:v>
+      </x:c>
+      <x:c r="H18" s="18" t="str">
+        <x:v>yearly 子范围同参一致</x:v>
+      </x:c>
+      <x:c r="I18" s="18" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="J18" s="18" t="str">
+        <x:v>docs/evidence/query_kline_year_live.md</x:v>
+      </x:c>
+      <x:c r="K18" s="18" t="str">
+        <x:v>LIVE_ALIGNED(yearly only)</x:v>
+      </x:c>
+      <x:c r="L18" s="18" t="str">
+        <x:v>分钟族未验且显式拒绝；年线线上单包样本；跨年多包仅合成覆盖</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="38" customHeight="1">
+      <x:c r="A19" s="18" t="str">
+        <x:v>B-20260826-15</x:v>
+      </x:c>
+      <x:c r="B19" s="18" t="str">
+        <x:v>2026-08-26</x:v>
+      </x:c>
+      <x:c r="C19" s="18" t="str">
+        <x:v>QuerySecuritiesInfo</x:v>
+      </x:c>
+      <x:c r="D19" s="18" t="str">
+        <x:v>SSE 510300 单代码最小只读闭环</x:v>
+      </x:c>
+      <x:c r="E19" s="18" t="str">
+        <x:v>盘后查询</x:v>
+      </x:c>
+      <x:c r="F19" s="18" t="str">
+        <x:v>login true、error 0、1行/43列（int/str）、market=[101]、variety=[2]；wire: push ReqGetCodeTableList/Security=510300|101/tag=字符串109/ReqGetCodelistComplete</x:v>
+      </x:c>
+      <x:c r="G19" s="18" t="str">
+        <x:v>error 0、1 行、43 列类型/不变量与 Linux 逐项一致</x:v>
+      </x:c>
+      <x:c r="H19" s="18" t="str">
+        <x:v>SSE single code 子范围同参一致</x:v>
+      </x:c>
+      <x:c r="I19" s="18" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="J19" s="18" t="str">
+        <x:v>docs/evidence/query_securities_info_sse.md</x:v>
+      </x:c>
+      <x:c r="K19" s="18" t="str">
+        <x:v>LIVE_ALIGNED(SSE single code only)</x:v>
+      </x:c>
+      <x:c r="L19" s="18" t="str">
+        <x:v>全市场/多item/SZSE/NEEQ 显式拒绝；空结果/非零status未取证；push 无重连</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="38" customHeight="1">
+      <x:c r="A20" s="18" t="str">
+        <x:v>B-20260826-16</x:v>
+      </x:c>
+      <x:c r="B20" s="18" t="str">
+        <x:v>2026-08-26</x:v>
+      </x:c>
+      <x:c r="C20" s="18" t="str">
+        <x:v>QueryExFactorTable</x:v>
+      </x:c>
+      <x:c r="D20" s="18" t="str">
+        <x:v>000001 单代码最小只读闭环</x:v>
+      </x:c>
+      <x:c r="E20" s="18" t="str">
+        <x:v>盘后查询</x:v>
+      </x:c>
+      <x:c r="F20" s="18" t="str">
+        <x:v>login true、err 0、33行/5列（inner_code/code str、ex_date int、ex_factor/cum_factor float）、double 18位往返无损、cum_factor 单调违例2处；wire: dgw1_query ReqGetExFactor/tag=11102/5字段CSV/ReqGetComplete</x:v>
+      </x:c>
+      <x:c r="G20" s="18" t="str">
+        <x:v>err 0、33 行、5 列类型/不变量与 Linux 逐项一致（含单调违例2处吻合）</x:v>
+      </x:c>
+      <x:c r="H20" s="18" t="str">
+        <x:v>000001 子范围同参一致</x:v>
+      </x:c>
+      <x:c r="I20" s="18" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="J20" s="18" t="str">
+        <x:v>docs/evidence/query_ex_factor_table_000001.md</x:v>
+      </x:c>
+      <x:c r="K20" s="18" t="str">
+        <x:v>LIVE_ALIGNED(000001 only)</x:v>
+      </x:c>
+      <x:c r="L20" s="18" t="str">
+        <x:v>空结果/非零status未取证；多包未线上观测；异步 SPI 未实现；double 缩放按 N38(15) 由调用方处理</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="38" customHeight="1">
+      <x:c r="A21" s="22" t="str">
         <x:v>后续 Agent 每次追加一行；一项接口/一个明确子范围/一个批次</x:v>
       </x:c>
-      <x:c r="B14" s="22" t="str">
+      <x:c r="B21" s="22" t="str">
         <x:v>后续 Agent 每次追加一行；一项接口/一个明确子范围/一个批次</x:v>
       </x:c>
-      <x:c r="C14" s="22" t="str">
+      <x:c r="C21" s="22" t="str">
         <x:v>后续 Agent 每次追加一行；一项接口/一个明确子范围/一个批次</x:v>
       </x:c>
-      <x:c r="D14" s="22" t="str">
+      <x:c r="D21" s="22" t="str">
         <x:v>后续 Agent 每次追加一行；一项接口/一个明确子范围/一个批次</x:v>
       </x:c>
-      <x:c r="E14" s="22" t="str">
+      <x:c r="E21" s="22" t="str">
         <x:v>后续 Agent 每次追加一行；一项接口/一个明确子范围/一个批次</x:v>
       </x:c>
-      <x:c r="F14" s="22" t="str">
+      <x:c r="F21" s="22" t="str">
         <x:v>后续 Agent 每次追加一行；一项接口/一个明确子范围/一个批次</x:v>
       </x:c>
-      <x:c r="G14" s="22" t="str">
+      <x:c r="G21" s="22" t="str">
         <x:v>后续 Agent 每次追加一行；一项接口/一个明确子范围/一个批次</x:v>
       </x:c>
-      <x:c r="H14" s="22" t="str">
+      <x:c r="H21" s="22" t="str">
         <x:v>后续 Agent 每次追加一行；一项接口/一个明确子范围/一个批次</x:v>
       </x:c>
-      <x:c r="I14" s="22" t="str">
+      <x:c r="I21" s="22" t="str">
         <x:v>后续 Agent 每次追加一行；一项接口/一个明确子范围/一个批次</x:v>
       </x:c>
-      <x:c r="J14" s="22" t="str">
+      <x:c r="J21" s="22" t="str">
         <x:v>后续 Agent 每次追加一行；一项接口/一个明确子范围/一个批次</x:v>
       </x:c>
-      <x:c r="K14" s="22" t="str">
+      <x:c r="K21" s="22" t="str">
         <x:v>后续 Agent 每次追加一行；一项接口/一个明确子范围/一个批次</x:v>
       </x:c>
-      <x:c r="L14" s="22" t="str">
+      <x:c r="L21" s="22" t="str">
         <x:v>后续 Agent 每次追加一行；一项接口/一个明确子范围/一个批次</x:v>
       </x:c>
-    </x:row>
-    <x:row r="15" ht="38" customHeight="1">
-      <x:c r="A15" s="18" t="str"/>
-      <x:c r="B15" s="18" t="str"/>
-      <x:c r="C15" s="18" t="str"/>
-      <x:c r="D15" s="18" t="str"/>
-      <x:c r="E15" s="18" t="str"/>
-      <x:c r="F15" s="18" t="str"/>
-      <x:c r="G15" s="18" t="str"/>
-      <x:c r="H15" s="18" t="str"/>
-      <x:c r="I15" s="18" t="str"/>
-      <x:c r="J15" s="18" t="str"/>
-      <x:c r="K15" s="18" t="str"/>
-      <x:c r="L15" s="18" t="str"/>
-    </x:row>
-    <x:row r="16" ht="38" customHeight="1">
-      <x:c r="A16" s="18" t="str"/>
-      <x:c r="B16" s="18" t="str"/>
-      <x:c r="C16" s="18" t="str"/>
-      <x:c r="D16" s="18" t="str"/>
-      <x:c r="E16" s="18" t="str"/>
-      <x:c r="F16" s="18" t="str"/>
-      <x:c r="G16" s="18" t="str"/>
-      <x:c r="H16" s="18" t="str"/>
-      <x:c r="I16" s="18" t="str"/>
-      <x:c r="J16" s="18" t="str"/>
-      <x:c r="K16" s="18" t="str"/>
-      <x:c r="L16" s="18" t="str"/>
-    </x:row>
-    <x:row r="17" ht="38" customHeight="1">
-      <x:c r="A17" s="18" t="str"/>
-      <x:c r="B17" s="18" t="str"/>
-      <x:c r="C17" s="18" t="str"/>
-      <x:c r="D17" s="18" t="str"/>
-      <x:c r="E17" s="18" t="str"/>
-      <x:c r="F17" s="18" t="str"/>
-      <x:c r="G17" s="18" t="str"/>
-      <x:c r="H17" s="18" t="str"/>
-      <x:c r="I17" s="18" t="str"/>
-      <x:c r="J17" s="18" t="str"/>
-      <x:c r="K17" s="18" t="str"/>
-      <x:c r="L17" s="18" t="str"/>
-    </x:row>
-    <x:row r="18" ht="38" customHeight="1">
-      <x:c r="A18" s="18" t="str"/>
-      <x:c r="B18" s="18" t="str"/>
-      <x:c r="C18" s="18" t="str"/>
-      <x:c r="D18" s="18" t="str"/>
-      <x:c r="E18" s="18" t="str"/>
-      <x:c r="F18" s="18" t="str"/>
-      <x:c r="G18" s="18" t="str"/>
-      <x:c r="H18" s="18" t="str"/>
-      <x:c r="I18" s="18" t="str"/>
-      <x:c r="J18" s="18" t="str"/>
-      <x:c r="K18" s="18" t="str"/>
-      <x:c r="L18" s="18" t="str"/>
-    </x:row>
-    <x:row r="19" ht="38" customHeight="1">
-      <x:c r="A19" s="18" t="str"/>
-      <x:c r="B19" s="18" t="str"/>
-      <x:c r="C19" s="18" t="str"/>
-      <x:c r="D19" s="18" t="str"/>
-      <x:c r="E19" s="18" t="str"/>
-      <x:c r="F19" s="18" t="str"/>
-      <x:c r="G19" s="18" t="str"/>
-      <x:c r="H19" s="18" t="str"/>
-      <x:c r="I19" s="18" t="str"/>
-      <x:c r="J19" s="18" t="str"/>
-      <x:c r="K19" s="18" t="str"/>
-      <x:c r="L19" s="18" t="str"/>
-    </x:row>
-    <x:row r="20" ht="38" customHeight="1">
-      <x:c r="A20" s="18" t="str"/>
-      <x:c r="B20" s="18" t="str"/>
-      <x:c r="C20" s="18" t="str"/>
-      <x:c r="D20" s="18" t="str"/>
-      <x:c r="E20" s="18" t="str"/>
-      <x:c r="F20" s="18" t="str"/>
-      <x:c r="G20" s="18" t="str"/>
-      <x:c r="H20" s="18" t="str"/>
-      <x:c r="I20" s="18" t="str"/>
-      <x:c r="J20" s="18" t="str"/>
-      <x:c r="K20" s="18" t="str"/>
-      <x:c r="L20" s="18" t="str"/>
-    </x:row>
-    <x:row r="21" ht="38" customHeight="1">
-      <x:c r="A21" s="18" t="str"/>
-      <x:c r="B21" s="18" t="str"/>
-      <x:c r="C21" s="18" t="str"/>
-      <x:c r="D21" s="18" t="str"/>
-      <x:c r="E21" s="18" t="str"/>
-      <x:c r="F21" s="18" t="str"/>
-      <x:c r="G21" s="18" t="str"/>
-      <x:c r="H21" s="18" t="str"/>
-      <x:c r="I21" s="18" t="str"/>
-      <x:c r="J21" s="18" t="str"/>
-      <x:c r="K21" s="18" t="str"/>
-      <x:c r="L21" s="18" t="str"/>
     </x:row>
     <x:row r="22" ht="38" customHeight="1">
       <x:c r="A22" s="18" t="str"/>
@@ -15353,17 +15531,115 @@
       <x:c r="K23" s="18" t="str"/>
       <x:c r="L23" s="18" t="str"/>
     </x:row>
+    <x:row r="24" ht="38" customHeight="1">
+      <x:c r="A24" s="18" t="str"/>
+      <x:c r="B24" s="18" t="str"/>
+      <x:c r="C24" s="18" t="str"/>
+      <x:c r="D24" s="18" t="str"/>
+      <x:c r="E24" s="18" t="str"/>
+      <x:c r="F24" s="18" t="str"/>
+      <x:c r="G24" s="18" t="str"/>
+      <x:c r="H24" s="18" t="str"/>
+      <x:c r="I24" s="18" t="str"/>
+      <x:c r="J24" s="18" t="str"/>
+      <x:c r="K24" s="18" t="str"/>
+      <x:c r="L24" s="18" t="str"/>
+    </x:row>
+    <x:row r="25" ht="38" customHeight="1">
+      <x:c r="A25" s="18" t="str"/>
+      <x:c r="B25" s="18" t="str"/>
+      <x:c r="C25" s="18" t="str"/>
+      <x:c r="D25" s="18" t="str"/>
+      <x:c r="E25" s="18" t="str"/>
+      <x:c r="F25" s="18" t="str"/>
+      <x:c r="G25" s="18" t="str"/>
+      <x:c r="H25" s="18" t="str"/>
+      <x:c r="I25" s="18" t="str"/>
+      <x:c r="J25" s="18" t="str"/>
+      <x:c r="K25" s="18" t="str"/>
+      <x:c r="L25" s="18" t="str"/>
+    </x:row>
+    <x:row r="26" ht="38" customHeight="1">
+      <x:c r="A26" s="18" t="str"/>
+      <x:c r="B26" s="18" t="str"/>
+      <x:c r="C26" s="18" t="str"/>
+      <x:c r="D26" s="18" t="str"/>
+      <x:c r="E26" s="18" t="str"/>
+      <x:c r="F26" s="18" t="str"/>
+      <x:c r="G26" s="18" t="str"/>
+      <x:c r="H26" s="18" t="str"/>
+      <x:c r="I26" s="18" t="str"/>
+      <x:c r="J26" s="18" t="str"/>
+      <x:c r="K26" s="18" t="str"/>
+      <x:c r="L26" s="18" t="str"/>
+    </x:row>
+    <x:row r="27" ht="38" customHeight="1">
+      <x:c r="A27" s="18" t="str"/>
+      <x:c r="B27" s="18" t="str"/>
+      <x:c r="C27" s="18" t="str"/>
+      <x:c r="D27" s="18" t="str"/>
+      <x:c r="E27" s="18" t="str"/>
+      <x:c r="F27" s="18" t="str"/>
+      <x:c r="G27" s="18" t="str"/>
+      <x:c r="H27" s="18" t="str"/>
+      <x:c r="I27" s="18" t="str"/>
+      <x:c r="J27" s="18" t="str"/>
+      <x:c r="K27" s="18" t="str"/>
+      <x:c r="L27" s="18" t="str"/>
+    </x:row>
+    <x:row r="28" ht="38" customHeight="1">
+      <x:c r="A28" s="18" t="str"/>
+      <x:c r="B28" s="18" t="str"/>
+      <x:c r="C28" s="18" t="str"/>
+      <x:c r="D28" s="18" t="str"/>
+      <x:c r="E28" s="18" t="str"/>
+      <x:c r="F28" s="18" t="str"/>
+      <x:c r="G28" s="18" t="str"/>
+      <x:c r="H28" s="18" t="str"/>
+      <x:c r="I28" s="18" t="str"/>
+      <x:c r="J28" s="18" t="str"/>
+      <x:c r="K28" s="18" t="str"/>
+      <x:c r="L28" s="18" t="str"/>
+    </x:row>
+    <x:row r="29" ht="38" customHeight="1">
+      <x:c r="A29" s="18" t="str"/>
+      <x:c r="B29" s="18" t="str"/>
+      <x:c r="C29" s="18" t="str"/>
+      <x:c r="D29" s="18" t="str"/>
+      <x:c r="E29" s="18" t="str"/>
+      <x:c r="F29" s="18" t="str"/>
+      <x:c r="G29" s="18" t="str"/>
+      <x:c r="H29" s="18" t="str"/>
+      <x:c r="I29" s="18" t="str"/>
+      <x:c r="J29" s="18" t="str"/>
+      <x:c r="K29" s="18" t="str"/>
+      <x:c r="L29" s="18" t="str"/>
+    </x:row>
+    <x:row r="30" ht="38" customHeight="1">
+      <x:c r="A30" s="18" t="str"/>
+      <x:c r="B30" s="18" t="str"/>
+      <x:c r="C30" s="18" t="str"/>
+      <x:c r="D30" s="18" t="str"/>
+      <x:c r="E30" s="18" t="str"/>
+      <x:c r="F30" s="18" t="str"/>
+      <x:c r="G30" s="18" t="str"/>
+      <x:c r="H30" s="18" t="str"/>
+      <x:c r="I30" s="18" t="str"/>
+      <x:c r="J30" s="18" t="str"/>
+      <x:c r="K30" s="18" t="str"/>
+      <x:c r="L30" s="18" t="str"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:L1"/>
     <x:mergeCell ref="A2:L2"/>
-    <x:mergeCell ref="A14:L14"/>
+    <x:mergeCell ref="A21:L21"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="I5:I23">
+    <x:dataValidation type="list" sqref="I5:I30">
       <x:formula1>"是,否"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="K5:K23">
+    <x:dataValidation type="list" sqref="K5:K30">
       <x:formula1>'状态字典'!$A$5:$A$16</x:formula1>
     </x:dataValidation>
   </x:dataValidations>

</xml_diff>